<commit_message>
Add measured mass, centre of gravity and tyre geometry
- Chapter 1: mass, axle loads and CoG from the scales and tilt test
  (T01/T02, without body), tyre diameters and runout (T12), wheel mass
  (T17), camera and holder mass, tipping limit from the measured CoG
- Chapters 0 and 4: measured mass and CoG instead of placeholders
- Workbook: measured values entered, unmeasured placeholders removed,
  self-steer radius formula corrected (R = T*d/delta_d)
- Iteration figure: regional robot no longer cut off on the left
</commit_message>
<xml_diff>
--- a/docs/data/manual/mobility_measurements.xlsx
+++ b/docs/data/manual/mobility_measurements.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Grip_Tipping" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Step_Log" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -2099,7 +2099,7 @@
     <t xml:space="preserve">Ø difference rear left − right [mm]</t>
   </si>
   <si>
-    <t xml:space="preserve">Resulting self-steer radius of the rear axle R = T·d/(2·Δd) [m]</t>
+    <t xml:space="preserve">Resulting self-steer radius of the rear axle R = T·d/Δd [m]</t>
   </si>
   <si>
     <t xml:space="preserve">Lateral deviation after 3 m straight run, measured [mm]</t>
@@ -13705,9 +13705,7 @@
         <f aca="false">G15-$B$7</f>
         <v>36.98</v>
       </c>
-      <c r="K15" s="19" t="n">
-        <v>105</v>
-      </c>
+      <c r="K15" s="19"/>
       <c r="L15" s="25" t="n">
         <f aca="false">IF(K15="","",K15*H15)</f>
         <v>11648.7</v>
@@ -13759,9 +13757,7 @@
         <f aca="false">G16-$B$7</f>
         <v>15.45</v>
       </c>
-      <c r="K16" s="19" t="n">
-        <v>21</v>
-      </c>
+      <c r="K16" s="19"/>
       <c r="L16" s="25" t="n">
         <f aca="false">IF(K16="","",K16*H16)</f>
         <v>2488.29</v>
@@ -13813,9 +13809,7 @@
         <f aca="false">G17-$B$7</f>
         <v>15.09</v>
       </c>
-      <c r="K17" s="19" t="n">
-        <v>8.4</v>
-      </c>
+      <c r="K17" s="19"/>
       <c r="L17" s="25" t="n">
         <f aca="false">IF(K17="","",K17*H17)</f>
         <v>1020.936</v>
@@ -13867,9 +13861,7 @@
         <f aca="false">G18-$B$7</f>
         <v>15.35</v>
       </c>
-      <c r="K18" s="19" t="n">
-        <v>1.6</v>
-      </c>
+      <c r="K18" s="19"/>
       <c r="L18" s="25" t="n">
         <f aca="false">IF(K18="","",K18*H18)</f>
         <v>159.888</v>
@@ -13921,9 +13913,7 @@
         <f aca="false">G19-$B$7</f>
         <v>15.35</v>
       </c>
-      <c r="K19" s="19" t="n">
-        <v>1.6</v>
-      </c>
+      <c r="K19" s="19"/>
       <c r="L19" s="25" t="n">
         <f aca="false">IF(K19="","",K19*H19)</f>
         <v>159.872</v>
@@ -13975,9 +13965,7 @@
         <f aca="false">G20-$B$7</f>
         <v>18.99</v>
       </c>
-      <c r="K20" s="19" t="n">
-        <v>4.1</v>
-      </c>
+      <c r="K20" s="19"/>
       <c r="L20" s="25" t="n">
         <f aca="false">IF(K20="","",K20*H20)</f>
         <v>345.63</v>
@@ -14029,9 +14017,7 @@
         <f aca="false">G21-$B$7</f>
         <v>9.94</v>
       </c>
-      <c r="K21" s="19" t="n">
-        <v>0.3</v>
-      </c>
+      <c r="K21" s="19"/>
       <c r="L21" s="25" t="n">
         <f aca="false">IF(K21="","",K21*H21)</f>
         <v>31.221</v>
@@ -14083,9 +14069,7 @@
         <f aca="false">G22-$B$7</f>
         <v>5.82</v>
       </c>
-      <c r="K22" s="19" t="n">
-        <v>1.9</v>
-      </c>
+      <c r="K22" s="19"/>
       <c r="L22" s="25" t="n">
         <f aca="false">IF(K22="","",K22*H22)</f>
         <v>183.578</v>
@@ -14137,9 +14121,7 @@
         <f aca="false">G23-$B$7</f>
         <v>9.84</v>
       </c>
-      <c r="K23" s="19" t="n">
-        <v>1.9</v>
-      </c>
+      <c r="K23" s="19"/>
       <c r="L23" s="25" t="n">
         <f aca="false">IF(K23="","",K23*H23)</f>
         <v>169.385</v>
@@ -14191,9 +14173,7 @@
         <f aca="false">G24-$B$7</f>
         <v>7.83</v>
       </c>
-      <c r="K24" s="19" t="n">
-        <v>0.1</v>
-      </c>
+      <c r="K24" s="19"/>
       <c r="L24" s="25" t="n">
         <f aca="false">IF(K24="","",K24*H24)</f>
         <v>9.288</v>
@@ -14245,9 +14225,7 @@
         <f aca="false">G25-$B$7</f>
         <v>17.3</v>
       </c>
-      <c r="K25" s="19" t="n">
-        <v>1.5</v>
-      </c>
+      <c r="K25" s="19"/>
       <c r="L25" s="25" t="n">
         <f aca="false">IF(K25="","",K25*H25)</f>
         <v>214.275</v>
@@ -14299,9 +14277,7 @@
         <f aca="false">G26-$B$7</f>
         <v>15.18</v>
       </c>
-      <c r="K26" s="19" t="n">
-        <v>7.6</v>
-      </c>
+      <c r="K26" s="19"/>
       <c r="L26" s="25" t="n">
         <f aca="false">IF(K26="","",K26*H26)</f>
         <v>775.2</v>
@@ -14353,9 +14329,7 @@
         <f aca="false">G27-$B$7</f>
         <v>15.18</v>
       </c>
-      <c r="K27" s="19" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="K27" s="19"/>
       <c r="L27" s="25" t="n">
         <f aca="false">IF(K27="","",K27*H27)</f>
         <v>764.775</v>
@@ -14407,9 +14381,7 @@
         <f aca="false">G28-$B$7</f>
         <v>13.2</v>
       </c>
-      <c r="K28" s="19" t="n">
-        <v>3.4</v>
-      </c>
+      <c r="K28" s="19"/>
       <c r="L28" s="25" t="n">
         <f aca="false">IF(K28="","",K28*H28)</f>
         <v>336.226</v>
@@ -14461,9 +14433,7 @@
         <f aca="false">G29-$B$7</f>
         <v>34.06</v>
       </c>
-      <c r="K29" s="19" t="n">
-        <v>38</v>
-      </c>
+      <c r="K29" s="19"/>
       <c r="L29" s="25" t="n">
         <f aca="false">IF(K29="","",K29*H29)</f>
         <v>1393.46</v>
@@ -14515,9 +14485,7 @@
         <f aca="false">G30-$B$7</f>
         <v>18.56</v>
       </c>
-      <c r="K30" s="19" t="n">
-        <v>62</v>
-      </c>
+      <c r="K30" s="19"/>
       <c r="L30" s="25" t="n">
         <f aca="false">IF(K30="","",K30*H30)</f>
         <v>2367.16</v>
@@ -14569,9 +14537,7 @@
         <f aca="false">G31-$B$7</f>
         <v>46.23</v>
       </c>
-      <c r="K31" s="19" t="n">
-        <v>19</v>
-      </c>
+      <c r="K31" s="19"/>
       <c r="L31" s="25" t="n">
         <f aca="false">IF(K31="","",K31*H31)</f>
         <v>806.55</v>
@@ -14623,9 +14589,7 @@
         <f aca="false">G32-$B$7</f>
         <v>15.6</v>
       </c>
-      <c r="K32" s="19" t="n">
-        <v>94</v>
-      </c>
+      <c r="K32" s="19"/>
       <c r="L32" s="25" t="n">
         <f aca="false">IF(K32="","",K32*H32)</f>
         <v>4065.5</v>
@@ -14677,9 +14641,7 @@
         <f aca="false">G33-$B$7</f>
         <v>15.6</v>
       </c>
-      <c r="K33" s="19" t="n">
-        <v>2.6</v>
-      </c>
+      <c r="K33" s="19"/>
       <c r="L33" s="25" t="n">
         <f aca="false">IF(K33="","",K33*H33)</f>
         <v>19.812</v>
@@ -14731,9 +14693,7 @@
         <f aca="false">G34-$B$7</f>
         <v>16.06</v>
       </c>
-      <c r="K34" s="19" t="n">
-        <v>3</v>
-      </c>
+      <c r="K34" s="19"/>
       <c r="L34" s="25" t="n">
         <f aca="false">IF(K34="","",K34*H34)</f>
         <v>-0.0600000000000307</v>
@@ -14785,9 +14745,7 @@
         <f aca="false">G35-$B$7</f>
         <v>15.87</v>
       </c>
-      <c r="K35" s="19" t="n">
-        <v>4.6</v>
-      </c>
+      <c r="K35" s="19"/>
       <c r="L35" s="25" t="n">
         <f aca="false">IF(K35="","",K35*H35)</f>
         <v>-0.0920000000000471</v>
@@ -14839,9 +14797,7 @@
         <f aca="false">G36-$B$7</f>
         <v>41.93</v>
       </c>
-      <c r="K36" s="19" t="n">
-        <v>55</v>
-      </c>
+      <c r="K36" s="19"/>
       <c r="L36" s="25" t="n">
         <f aca="false">IF(K36="","",K36*H36)</f>
         <v>364.65</v>
@@ -14893,9 +14849,7 @@
         <f aca="false">G37-$B$7</f>
         <v>6.49</v>
       </c>
-      <c r="K37" s="19" t="n">
-        <v>3</v>
-      </c>
+      <c r="K37" s="19"/>
       <c r="L37" s="25" t="n">
         <f aca="false">IF(K37="","",K37*H37)</f>
         <v>-9.87000000000002</v>
@@ -14947,9 +14901,7 @@
         <f aca="false">G38-$B$7</f>
         <v>9.31</v>
       </c>
-      <c r="K38" s="19" t="n">
-        <v>21.3</v>
-      </c>
+      <c r="K38" s="19"/>
       <c r="L38" s="25" t="n">
         <f aca="false">IF(K38="","",K38*H38)</f>
         <v>1335.723</v>
@@ -15001,9 +14953,7 @@
         <f aca="false">G39-$B$7</f>
         <v>16.03</v>
       </c>
-      <c r="K39" s="19" t="n">
-        <v>9.4</v>
-      </c>
+      <c r="K39" s="19"/>
       <c r="L39" s="25" t="n">
         <f aca="false">IF(K39="","",K39*H39)</f>
         <v>-0.188000000000096</v>
@@ -15055,9 +15005,7 @@
         <f aca="false">G40-$B$7</f>
         <v>16.03</v>
       </c>
-      <c r="K40" s="19" t="n">
-        <v>9.5</v>
-      </c>
+      <c r="K40" s="19"/>
       <c r="L40" s="25" t="n">
         <f aca="false">IF(K40="","",K40*H40)</f>
         <v>7.21999999999991</v>
@@ -15109,9 +15057,7 @@
         <f aca="false">G41-$B$7</f>
         <v>15.6</v>
       </c>
-      <c r="K41" s="19" t="n">
-        <v>1.7</v>
-      </c>
+      <c r="K41" s="19"/>
       <c r="L41" s="25" t="n">
         <f aca="false">IF(K41="","",K41*H41)</f>
         <v>27.2</v>
@@ -15163,8 +15109,8 @@
         <f aca="false">G42-$B$7</f>
         <v>72.6</v>
       </c>
-      <c r="K42" s="19" t="n">
-        <v>30</v>
+      <c r="K42" s="19">
+        <v>23.05</v>
       </c>
       <c r="L42" s="25" t="n">
         <f aca="false">IF(K42="","",K42*H42)</f>
@@ -15217,9 +15163,7 @@
         <f aca="false">G43-$B$7</f>
         <v>45.7</v>
       </c>
-      <c r="K43" s="19" t="n">
-        <v>38</v>
-      </c>
+      <c r="K43" s="19"/>
       <c r="L43" s="25" t="n">
         <f aca="false">IF(K43="","",K43*H43)</f>
         <v>2283.8</v>
@@ -15265,9 +15209,7 @@
         <f aca="false">IF(G44="","",G44-$B$7)</f>
         <v>49.4</v>
       </c>
-      <c r="K44" s="19" t="n">
-        <v>16</v>
-      </c>
+      <c r="K44" s="19"/>
       <c r="L44" s="25" t="n">
         <f aca="false">IF(OR(K44="",H44=""),"",K44*H44)</f>
         <v>617.6</v>
@@ -15375,56 +15317,56 @@
       <c r="A55" s="18" t="s">
         <v>437</v>
       </c>
-      <c r="B55" s="19" t="n">
-        <v>575.3</v>
+      <c r="B55" s="19">
+        <v>586</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="18" t="s">
         <v>438</v>
       </c>
-      <c r="B56" s="19" t="n">
-        <v>335.7</v>
+      <c r="B56" s="19">
+        <v>322</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="18" t="s">
         <v>439</v>
       </c>
-      <c r="B57" s="19" t="n">
-        <v>240</v>
+      <c r="B57" s="19">
+        <v>257</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="18" t="s">
         <v>440</v>
       </c>
-      <c r="B58" s="19" t="n">
-        <v>303.7</v>
+      <c r="B58" s="19">
+        <v>284</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="18" t="s">
         <v>441</v>
       </c>
-      <c r="B59" s="19" t="n">
-        <v>271.3</v>
+      <c r="B59" s="19">
+        <v>295</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="18" t="s">
         <v>442</v>
       </c>
-      <c r="B60" s="19" t="n">
-        <v>25</v>
+      <c r="B60" s="19">
+        <v>40</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="18" t="s">
         <v>443</v>
       </c>
-      <c r="B61" s="19" t="n">
-        <v>357.5</v>
+      <c r="B61" s="19">
+        <v>377</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20280,14 +20222,14 @@
       <c r="A35" s="18" t="s">
         <v>640</v>
       </c>
-      <c r="B35" s="34" t="n">
-        <v>32.07</v>
-      </c>
-      <c r="C35" s="34" t="n">
-        <v>32.04</v>
-      </c>
-      <c r="D35" s="34" t="n">
-        <v>32.02</v>
+      <c r="B35" s="34">
+        <v>31.6</v>
+      </c>
+      <c r="C35" s="34">
+        <v>32.0</v>
+      </c>
+      <c r="D35" s="34">
+        <v>31.9</v>
       </c>
       <c r="E35" s="30" t="n">
         <f aca="false">IF(COUNT(B35:D35)=0,"",AVERAGE(B35:D35))</f>
@@ -20297,22 +20239,22 @@
         <f aca="false">IF(COUNT(B35:D35)&lt;2,"",MAX(B35:D35)-MIN(B35:D35))</f>
         <v>0.0499999999999972</v>
       </c>
-      <c r="G35" s="19" t="n">
-        <v>9.6</v>
+      <c r="G35" s="19">
+        <v>9</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
         <v>641</v>
       </c>
-      <c r="B36" s="34" t="n">
-        <v>32</v>
-      </c>
-      <c r="C36" s="34" t="n">
-        <v>31.94</v>
-      </c>
-      <c r="D36" s="34" t="n">
-        <v>32.02</v>
+      <c r="B36" s="34">
+        <v>32.1</v>
+      </c>
+      <c r="C36" s="34">
+        <v>32.0</v>
+      </c>
+      <c r="D36" s="34">
+        <v>32.1</v>
       </c>
       <c r="E36" s="30" t="n">
         <f aca="false">IF(COUNT(B36:D36)=0,"",AVERAGE(B36:D36))</f>
@@ -20322,22 +20264,22 @@
         <f aca="false">IF(COUNT(B36:D36)&lt;2,"",MAX(B36:D36)-MIN(B36:D36))</f>
         <v>0.0800000000000019</v>
       </c>
-      <c r="G36" s="19" t="n">
-        <v>9.7</v>
+      <c r="G36" s="19">
+        <v>9</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
         <v>642</v>
       </c>
-      <c r="B37" s="34" t="n">
-        <v>32.05</v>
-      </c>
-      <c r="C37" s="34" t="n">
-        <v>32.04</v>
-      </c>
-      <c r="D37" s="34" t="n">
-        <v>32.01</v>
+      <c r="B37" s="34">
+        <v>32.1</v>
+      </c>
+      <c r="C37" s="34">
+        <v>31.7</v>
+      </c>
+      <c r="D37" s="34">
+        <v>32.0</v>
       </c>
       <c r="E37" s="30" t="n">
         <f aca="false">IF(COUNT(B37:D37)=0,"",AVERAGE(B37:D37))</f>
@@ -20347,22 +20289,22 @@
         <f aca="false">IF(COUNT(B37:D37)&lt;2,"",MAX(B37:D37)-MIN(B37:D37))</f>
         <v>0.0399999999999992</v>
       </c>
-      <c r="G37" s="19" t="n">
-        <v>9.4</v>
+      <c r="G37" s="19">
+        <v>9</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
         <v>643</v>
       </c>
-      <c r="B38" s="34" t="n">
-        <v>31.97</v>
-      </c>
-      <c r="C38" s="34" t="n">
-        <v>32.01</v>
-      </c>
-      <c r="D38" s="34" t="n">
-        <v>31.96</v>
+      <c r="B38" s="34">
+        <v>32.0</v>
+      </c>
+      <c r="C38" s="34">
+        <v>32.0</v>
+      </c>
+      <c r="D38" s="34">
+        <v>32.0</v>
       </c>
       <c r="E38" s="30" t="n">
         <f aca="false">IF(COUNT(B38:D38)=0,"",AVERAGE(B38:D38))</f>
@@ -20372,8 +20314,8 @@
         <f aca="false">IF(COUNT(B38:D38)&lt;2,"",MAX(B38:D38)-MIN(B38:D38))</f>
         <v>0.0499999999999972</v>
       </c>
-      <c r="G38" s="19" t="n">
-        <v>9.2</v>
+      <c r="G38" s="19">
+        <v>9</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -20390,7 +20332,7 @@
         <v>645</v>
       </c>
       <c r="E41" s="24" t="n">
-        <f aca="false">IF(OR(E40="",E40=0),"",C15*AVERAGE(E37:E38)/(2*ABS(E40))/1000)</f>
+        <f aca="false">IF(OR(E40="",E40=0),"",C15*AVERAGE(E37:E38)/ABS(E40)/1000)</f>
         <v>28.8660125000013</v>
       </c>
     </row>
@@ -20398,9 +20340,7 @@
       <c r="A42" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="E42" s="36" t="n">
-        <v>21</v>
-      </c>
+      <c r="E42" s="36"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="18" t="s">

</xml_diff>

<commit_message>
Add the measured static steering angles (T05)
Full lock reaches 36.9 deg bicycle-equivalent on both sides instead of the
45 deg of the CAD; the Ackermann share is 62 % left and 138 % right. Replace
the placeholder series in Steering_Target_Actual and compare the static
angles with the driven steering table. Also remove the resolved CAD TODO and
name the SC09 as a Waveshare servo.
</commit_message>
<xml_diff>
--- a/docs/data/manual/mobility_measurements.xlsx
+++ b/docs/data/manual/mobility_measurements.xlsx
@@ -3008,32 +3008,17 @@
               <c:f>5</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="9"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>-45</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-33.8</c:v>
+                  <c:v>-13.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-22.5</c:v>
+                  <c:v>13.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-11.2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>11.2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>22.5</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>33.8</c:v>
-                </c:pt>
-                <c:pt idx="8">
                   <c:v>45</c:v>
                 </c:pt>
               </c:numCache>
@@ -3044,33 +3029,18 @@
               <c:f>4</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="9"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>-45.0235640645852</c:v>
+                  <c:v>-36.892</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-37.4617899392916</c:v>
+                  <c:v>-12.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-24.8929299257228</c:v>
+                  <c:v>13.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-11.8132768176948</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>8.67149673626152</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>18.5929746775438</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>30.9575078375836</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>43.9067346050426</c:v>
+                  <c:v>36.926</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -15654,48 +15624,44 @@
         <v>-45</v>
       </c>
       <c r="D11" s="19" t="n">
-        <v>-36.1</v>
-      </c>
-      <c r="E11" s="19" t="n">
-        <v>-36.7</v>
-      </c>
+        <v>-30</v>
+      </c>
+      <c r="E11" s="19"/>
       <c r="F11" s="19" t="n">
-        <v>-57</v>
-      </c>
-      <c r="G11" s="19" t="n">
-        <v>-57.6</v>
-      </c>
+        <v>-47</v>
+      </c>
+      <c r="G11" s="19"/>
       <c r="H11" s="24" t="n">
         <f aca="false">IF(COUNT(D11:E11)=0,"",AVERAGE(D11:E11))</f>
-        <v>-36.4</v>
+        <v>-30</v>
       </c>
       <c r="I11" s="24" t="n">
         <f aca="false">IF(COUNT(F11:G11)=0,"",AVERAGE(F11:G11))</f>
-        <v>-57.3</v>
+        <v>-47</v>
       </c>
       <c r="J11" s="24" t="n">
         <f aca="false">IF(OR(H11="",I11=""),"",IF(ABS(H11+I11)&lt;0.05,0,DEGREES(ATAN(2/(1/TAN(RADIANS(H11))+1/TAN(RADIANS(I11)))))))</f>
-        <v>-45.0235640645852</v>
+        <v>-36.891574350270105</v>
       </c>
       <c r="K11" s="24" t="n">
         <f aca="false">IF(OR(J11="",C11=""),"",J11-C11)</f>
-        <v>-0.0235640645852087</v>
-      </c>
-      <c r="L11" s="24" t="n">
+        <v>8.108425649729895</v>
+      </c>
+      <c r="L11" s="24" t="str">
         <f aca="false">IF(COUNT(D11:E11)&lt;2,"",D11-E11)</f>
-        <v>0.600000000000001</v>
-      </c>
-      <c r="M11" s="24" t="n">
+        <v/>
+      </c>
+      <c r="M11" s="24" t="str">
         <f aca="false">IF(COUNT(F11:G11)&lt;2,"",F11-G11)</f>
-        <v>0.600000000000001</v>
+        <v/>
       </c>
       <c r="N11" s="24" t="n">
         <f aca="false">IF(OR(H11="",I11=""),"",IF(ABS(H11)&lt;0.05,0,SIGN(H11)*DEGREES(ATAN(1/(1/TAN(RADIANS(MAX(ABS(H11),ABS(I11))))+$B$6/$B$5)))))</f>
-        <v>-39.2632547996961</v>
+        <v>-33.4467966292934</v>
       </c>
       <c r="O11" s="24" t="n">
         <f aca="false">IF(N11="","",SIGN(H11)*MIN(ABS(H11),ABS(I11))-N11)</f>
-        <v>2.86325479969607</v>
+        <v>3.4467966292934022</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15703,54 +15669,50 @@
         <v>480</v>
       </c>
       <c r="B12" s="14" t="n">
-        <v>-75</v>
+        <v>-30</v>
       </c>
       <c r="C12" s="19" t="n">
-        <v>-33.8</v>
+        <v>-13.5</v>
       </c>
       <c r="D12" s="19" t="n">
-        <v>-32.1</v>
-      </c>
-      <c r="E12" s="19" t="n">
-        <v>-32.8</v>
-      </c>
+        <v>-12.5</v>
+      </c>
+      <c r="E12" s="19"/>
       <c r="F12" s="19" t="n">
-        <v>-43.7</v>
-      </c>
-      <c r="G12" s="19" t="n">
-        <v>-44.2</v>
-      </c>
+        <v>-12.5</v>
+      </c>
+      <c r="G12" s="19"/>
       <c r="H12" s="24" t="n">
         <f aca="false">IF(COUNT(D12:E12)=0,"",AVERAGE(D12:E12))</f>
-        <v>-32.45</v>
+        <v>-12.5</v>
       </c>
       <c r="I12" s="24" t="n">
         <f aca="false">IF(COUNT(F12:G12)=0,"",AVERAGE(F12:G12))</f>
-        <v>-43.95</v>
+        <v>-12.5</v>
       </c>
       <c r="J12" s="24" t="n">
         <f aca="false">IF(OR(H12="",I12=""),"",IF(ABS(H12+I12)&lt;0.05,0,DEGREES(ATAN(2/(1/TAN(RADIANS(H12))+1/TAN(RADIANS(I12)))))))</f>
-        <v>-37.4617899392916</v>
+        <v>-12.500000000000002</v>
       </c>
       <c r="K12" s="24" t="n">
         <f aca="false">IF(OR(J12="",C12=""),"",J12-C12)</f>
-        <v>-3.66178993929158</v>
-      </c>
-      <c r="L12" s="24" t="n">
+        <v>0.9999999999999982</v>
+      </c>
+      <c r="L12" s="24" t="str">
         <f aca="false">IF(COUNT(D12:E12)&lt;2,"",D12-E12)</f>
-        <v>0.699999999999996</v>
-      </c>
-      <c r="M12" s="24" t="n">
+        <v/>
+      </c>
+      <c r="M12" s="24" t="str">
         <f aca="false">IF(COUNT(F12:G12)&lt;2,"",F12-G12)</f>
-        <v>0.5</v>
+        <v/>
       </c>
       <c r="N12" s="24" t="n">
         <f aca="false">IF(OR(H12="",I12=""),"",IF(ABS(H12)&lt;0.05,0,SIGN(H12)*DEGREES(ATAN(1/(1/TAN(RADIANS(MAX(ABS(H12),ABS(I12))))+$B$6/$B$5)))))</f>
-        <v>-31.7067256605011</v>
+        <v>-11.110546472846867</v>
       </c>
       <c r="O12" s="24" t="n">
         <f aca="false">IF(N12="","",SIGN(H12)*MIN(ABS(H12),ABS(I12))-N12)</f>
-        <v>-0.743274339498864</v>
+        <v>-1.3894535271531332</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15758,54 +15720,50 @@
         <v>481</v>
       </c>
       <c r="B13" s="14" t="n">
-        <v>-50</v>
+        <v>30</v>
       </c>
       <c r="C13" s="19" t="n">
-        <v>-22.5</v>
+        <v>13.5</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>-22.7</v>
-      </c>
-      <c r="E13" s="19" t="n">
-        <v>-23.3</v>
-      </c>
+        <v>13.5</v>
+      </c>
+      <c r="E13" s="19"/>
       <c r="F13" s="19" t="n">
-        <v>-26.8</v>
-      </c>
-      <c r="G13" s="19" t="n">
-        <v>-27.4</v>
-      </c>
+        <v>13.5</v>
+      </c>
+      <c r="G13" s="19"/>
       <c r="H13" s="24" t="n">
         <f aca="false">IF(COUNT(D13:E13)=0,"",AVERAGE(D13:E13))</f>
-        <v>-23</v>
+        <v>13.5</v>
       </c>
       <c r="I13" s="24" t="n">
         <f aca="false">IF(COUNT(F13:G13)=0,"",AVERAGE(F13:G13))</f>
-        <v>-27.1</v>
+        <v>13.5</v>
       </c>
       <c r="J13" s="24" t="n">
         <f aca="false">IF(OR(H13="",I13=""),"",IF(ABS(H13+I13)&lt;0.05,0,DEGREES(ATAN(2/(1/TAN(RADIANS(H13))+1/TAN(RADIANS(I13)))))))</f>
-        <v>-24.8929299257228</v>
+        <v>13.5</v>
       </c>
       <c r="K13" s="24" t="n">
         <f aca="false">IF(OR(J13="",C13=""),"",J13-C13)</f>
-        <v>-2.39292992572275</v>
-      </c>
-      <c r="L13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="24" t="str">
         <f aca="false">IF(COUNT(D13:E13)&lt;2,"",D13-E13)</f>
-        <v>0.600000000000001</v>
-      </c>
-      <c r="M13" s="24" t="n">
+        <v/>
+      </c>
+      <c r="M13" s="24" t="str">
         <f aca="false">IF(COUNT(F13:G13)&lt;2,"",F13-G13)</f>
-        <v>0.599999999999998</v>
+        <v/>
       </c>
       <c r="N13" s="24" t="n">
         <f aca="false">IF(OR(H13="",I13=""),"",IF(ABS(H13)&lt;0.05,0,SIGN(H13)*DEGREES(ATAN(1/(1/TAN(RADIANS(MAX(ABS(H13),ABS(I13))))+$B$6/$B$5)))))</f>
-        <v>-21.523914162631</v>
+        <v>11.896755230393419</v>
       </c>
       <c r="O13" s="24" t="n">
         <f aca="false">IF(N13="","",SIGN(H13)*MIN(ABS(H13),ABS(I13))-N13)</f>
-        <v>-1.47608583736902</v>
+        <v>1.6032447696065812</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15813,329 +15771,265 @@
         <v>482</v>
       </c>
       <c r="B14" s="14" t="n">
-        <v>-25</v>
+        <v>100</v>
       </c>
       <c r="C14" s="19" t="n">
-        <v>-11.2</v>
+        <v>45</v>
       </c>
       <c r="D14" s="19" t="n">
-        <v>-11.2</v>
-      </c>
-      <c r="E14" s="19" t="n">
-        <v>-11.7</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="E14" s="19"/>
       <c r="F14" s="19" t="n">
-        <v>-11.9</v>
-      </c>
-      <c r="G14" s="19" t="n">
-        <v>-12.5</v>
-      </c>
+        <v>33.5</v>
+      </c>
+      <c r="G14" s="19"/>
       <c r="H14" s="24" t="n">
         <f aca="false">IF(COUNT(D14:E14)=0,"",AVERAGE(D14:E14))</f>
-        <v>-11.45</v>
+        <v>41</v>
       </c>
       <c r="I14" s="24" t="n">
         <f aca="false">IF(COUNT(F14:G14)=0,"",AVERAGE(F14:G14))</f>
-        <v>-12.2</v>
+        <v>33.5</v>
       </c>
       <c r="J14" s="24" t="n">
         <f aca="false">IF(OR(H14="",I14=""),"",IF(ABS(H14+I14)&lt;0.05,0,DEGREES(ATAN(2/(1/TAN(RADIANS(H14))+1/TAN(RADIANS(I14)))))))</f>
-        <v>-11.8132768176948</v>
+        <v>36.92631350724614</v>
       </c>
       <c r="K14" s="24" t="n">
         <f aca="false">IF(OR(J14="",C14=""),"",J14-C14)</f>
-        <v>-0.613276817694786</v>
-      </c>
-      <c r="L14" s="24" t="n">
+        <v>-8.073686492753858</v>
+      </c>
+      <c r="L14" s="24" t="str">
         <f aca="false">IF(COUNT(D14:E14)&lt;2,"",D14-E14)</f>
-        <v>0.5</v>
-      </c>
-      <c r="M14" s="24" t="n">
+        <v/>
+      </c>
+      <c r="M14" s="24" t="str">
         <f aca="false">IF(COUNT(F14:G14)&lt;2,"",F14-G14)</f>
-        <v>0.6</v>
+        <v/>
       </c>
       <c r="N14" s="24" t="n">
         <f aca="false">IF(OR(H14="",I14=""),"",IF(ABS(H14)&lt;0.05,0,SIGN(H14)*DEGREES(ATAN(1/(1/TAN(RADIANS(MAX(ABS(H14),ABS(I14))))+$B$6/$B$5)))))</f>
-        <v>-10.8721476127752</v>
+        <v>30.004438888901348</v>
       </c>
       <c r="O14" s="24" t="n">
         <f aca="false">IF(N14="","",SIGN(H14)*MIN(ABS(H14),ABS(I14))-N14)</f>
-        <v>-0.577852387224827</v>
+        <v>3.4955611110986524</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
         <v>483</v>
       </c>
-      <c r="B15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E15" s="19" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="F15" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G15" s="19" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="H15" s="24" t="n">
+      <c r="B15" s="14"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="24" t="str">
         <f aca="false">IF(COUNT(D15:E15)=0,"",AVERAGE(D15:E15))</f>
-        <v>0.2</v>
-      </c>
-      <c r="I15" s="24" t="n">
+        <v/>
+      </c>
+      <c r="I15" s="24" t="str">
         <f aca="false">IF(COUNT(F15:G15)=0,"",AVERAGE(F15:G15))</f>
-        <v>0.2</v>
-      </c>
-      <c r="J15" s="24" t="n">
+        <v/>
+      </c>
+      <c r="J15" s="24" t="str">
         <f aca="false">IF(OR(H15="",I15=""),"",IF(ABS(H15+I15)&lt;0.05,0,DEGREES(ATAN(2/(1/TAN(RADIANS(H15))+1/TAN(RADIANS(I15)))))))</f>
-        <v>0.2</v>
-      </c>
-      <c r="K15" s="24" t="n">
+        <v/>
+      </c>
+      <c r="K15" s="24" t="str">
         <f aca="false">IF(OR(J15="",C15=""),"",J15-C15)</f>
-        <v>0.2</v>
-      </c>
-      <c r="L15" s="24" t="n">
+        <v/>
+      </c>
+      <c r="L15" s="24" t="str">
         <f aca="false">IF(COUNT(D15:E15)&lt;2,"",D15-E15)</f>
-        <v>0.6</v>
-      </c>
-      <c r="M15" s="24" t="n">
+        <v/>
+      </c>
+      <c r="M15" s="24" t="str">
         <f aca="false">IF(COUNT(F15:G15)&lt;2,"",F15-G15)</f>
-        <v>0.6</v>
-      </c>
-      <c r="N15" s="24" t="n">
+        <v/>
+      </c>
+      <c r="N15" s="24" t="str">
         <f aca="false">IF(OR(H15="",I15=""),"",IF(ABS(H15)&lt;0.05,0,SIGN(H15)*DEGREES(ATAN(1/(1/TAN(RADIANS(MAX(ABS(H15),ABS(I15))))+$B$6/$B$5)))))</f>
-        <v>0.199594949034874</v>
-      </c>
-      <c r="O15" s="24" t="n">
+        <v/>
+      </c>
+      <c r="O15" s="24" t="str">
         <f aca="false">IF(N15="","",SIGN(H15)*MIN(ABS(H15),ABS(I15))-N15)</f>
-        <v>0.000405050965125664</v>
+        <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
         <v>484</v>
       </c>
-      <c r="B16" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="C16" s="19" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="D16" s="19" t="n">
-        <v>9.1</v>
-      </c>
-      <c r="E16" s="19" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="F16" s="19" t="n">
-        <v>8.8</v>
-      </c>
-      <c r="G16" s="19" t="n">
-        <v>8.2</v>
-      </c>
-      <c r="H16" s="24" t="n">
+      <c r="B16" s="14"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="24" t="str">
         <f aca="false">IF(COUNT(D16:E16)=0,"",AVERAGE(D16:E16))</f>
-        <v>8.85</v>
-      </c>
-      <c r="I16" s="24" t="n">
+        <v/>
+      </c>
+      <c r="I16" s="24" t="str">
         <f aca="false">IF(COUNT(F16:G16)=0,"",AVERAGE(F16:G16))</f>
-        <v>8.5</v>
-      </c>
-      <c r="J16" s="24" t="n">
+        <v/>
+      </c>
+      <c r="J16" s="24" t="str">
         <f aca="false">IF(OR(H16="",I16=""),"",IF(ABS(H16+I16)&lt;0.05,0,DEGREES(ATAN(2/(1/TAN(RADIANS(H16))+1/TAN(RADIANS(I16)))))))</f>
-        <v>8.67149673626152</v>
-      </c>
-      <c r="K16" s="24" t="n">
+        <v/>
+      </c>
+      <c r="K16" s="24" t="str">
         <f aca="false">IF(OR(J16="",C16=""),"",J16-C16)</f>
-        <v>-2.52850326373848</v>
-      </c>
-      <c r="L16" s="24" t="n">
+        <v/>
+      </c>
+      <c r="L16" s="24" t="str">
         <f aca="false">IF(COUNT(D16:E16)&lt;2,"",D16-E16)</f>
-        <v>0.5</v>
-      </c>
-      <c r="M16" s="24" t="n">
+        <v/>
+      </c>
+      <c r="M16" s="24" t="str">
         <f aca="false">IF(COUNT(F16:G16)&lt;2,"",F16-G16)</f>
-        <v>0.600000000000001</v>
-      </c>
-      <c r="N16" s="24" t="n">
+        <v/>
+      </c>
+      <c r="N16" s="24" t="str">
         <f aca="false">IF(OR(H16="",I16=""),"",IF(ABS(H16)&lt;0.05,0,SIGN(H16)*DEGREES(ATAN(1/(1/TAN(RADIANS(MAX(ABS(H16),ABS(I16))))+$B$6/$B$5)))))</f>
-        <v>8.12563270472141</v>
-      </c>
-      <c r="O16" s="24" t="n">
+        <v/>
+      </c>
+      <c r="O16" s="24" t="str">
         <f aca="false">IF(N16="","",SIGN(H16)*MIN(ABS(H16),ABS(I16))-N16)</f>
-        <v>0.374367295278592</v>
+        <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
         <v>485</v>
       </c>
-      <c r="B17" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="C17" s="19" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="D17" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="E17" s="19" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="F17" s="19" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="G17" s="19" t="n">
-        <v>17.3</v>
-      </c>
-      <c r="H17" s="24" t="n">
+      <c r="B17" s="14"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="24" t="str">
         <f aca="false">IF(COUNT(D17:E17)=0,"",AVERAGE(D17:E17))</f>
-        <v>19.7</v>
-      </c>
-      <c r="I17" s="24" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="24" t="str">
         <f aca="false">IF(COUNT(F17:G17)=0,"",AVERAGE(F17:G17))</f>
-        <v>17.6</v>
-      </c>
-      <c r="J17" s="24" t="n">
+        <v/>
+      </c>
+      <c r="J17" s="24" t="str">
         <f aca="false">IF(OR(H17="",I17=""),"",IF(ABS(H17+I17)&lt;0.05,0,DEGREES(ATAN(2/(1/TAN(RADIANS(H17))+1/TAN(RADIANS(I17)))))))</f>
-        <v>18.5929746775438</v>
-      </c>
-      <c r="K17" s="24" t="n">
+        <v/>
+      </c>
+      <c r="K17" s="24" t="str">
         <f aca="false">IF(OR(J17="",C17=""),"",J17-C17)</f>
-        <v>-3.90702532245617</v>
-      </c>
-      <c r="L17" s="24" t="n">
+        <v/>
+      </c>
+      <c r="L17" s="24" t="str">
         <f aca="false">IF(COUNT(D17:E17)&lt;2,"",D17-E17)</f>
-        <v>0.600000000000001</v>
-      </c>
-      <c r="M17" s="24" t="n">
+        <v/>
+      </c>
+      <c r="M17" s="24" t="str">
         <f aca="false">IF(COUNT(F17:G17)&lt;2,"",F17-G17)</f>
-        <v>0.599999999999998</v>
-      </c>
-      <c r="N17" s="24" t="n">
+        <v/>
+      </c>
+      <c r="N17" s="24" t="str">
         <f aca="false">IF(OR(H17="",I17=""),"",IF(ABS(H17)&lt;0.05,0,SIGN(H17)*DEGREES(ATAN(1/(1/TAN(RADIANS(MAX(ABS(H17),ABS(I17))))+$B$6/$B$5)))))</f>
-        <v>16.5077643294667</v>
-      </c>
-      <c r="O17" s="24" t="n">
+        <v/>
+      </c>
+      <c r="O17" s="24" t="str">
         <f aca="false">IF(N17="","",SIGN(H17)*MIN(ABS(H17),ABS(I17))-N17)</f>
-        <v>1.09223567053327</v>
+        <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
         <v>486</v>
       </c>
-      <c r="B18" s="14" t="n">
-        <v>75</v>
-      </c>
-      <c r="C18" s="19" t="n">
-        <v>33.8</v>
-      </c>
-      <c r="D18" s="19" t="n">
-        <v>35</v>
-      </c>
-      <c r="E18" s="19" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="F18" s="19" t="n">
-        <v>28.1</v>
-      </c>
-      <c r="G18" s="19" t="n">
-        <v>27.6</v>
-      </c>
-      <c r="H18" s="24" t="n">
+      <c r="B18" s="14"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="24" t="str">
         <f aca="false">IF(COUNT(D18:E18)=0,"",AVERAGE(D18:E18))</f>
-        <v>34.75</v>
-      </c>
-      <c r="I18" s="24" t="n">
+        <v/>
+      </c>
+      <c r="I18" s="24" t="str">
         <f aca="false">IF(COUNT(F18:G18)=0,"",AVERAGE(F18:G18))</f>
-        <v>27.85</v>
-      </c>
-      <c r="J18" s="24" t="n">
+        <v/>
+      </c>
+      <c r="J18" s="24" t="str">
         <f aca="false">IF(OR(H18="",I18=""),"",IF(ABS(H18+I18)&lt;0.05,0,DEGREES(ATAN(2/(1/TAN(RADIANS(H18))+1/TAN(RADIANS(I18)))))))</f>
-        <v>30.9575078375836</v>
-      </c>
-      <c r="K18" s="24" t="n">
+        <v/>
+      </c>
+      <c r="K18" s="24" t="str">
         <f aca="false">IF(OR(J18="",C18=""),"",J18-C18)</f>
-        <v>-2.8424921624164</v>
-      </c>
-      <c r="L18" s="24" t="n">
+        <v/>
+      </c>
+      <c r="L18" s="24" t="str">
         <f aca="false">IF(COUNT(D18:E18)&lt;2,"",D18-E18)</f>
-        <v>0.5</v>
-      </c>
-      <c r="M18" s="24" t="n">
+        <v/>
+      </c>
+      <c r="M18" s="24" t="str">
         <f aca="false">IF(COUNT(F18:G18)&lt;2,"",F18-G18)</f>
-        <v>0.5</v>
-      </c>
-      <c r="N18" s="24" t="n">
+        <v/>
+      </c>
+      <c r="N18" s="24" t="str">
         <f aca="false">IF(OR(H18="",I18=""),"",IF(ABS(H18)&lt;0.05,0,SIGN(H18)*DEGREES(ATAN(1/(1/TAN(RADIANS(MAX(ABS(H18),ABS(I18))))+$B$6/$B$5)))))</f>
-        <v>26.3053960961208</v>
-      </c>
-      <c r="O18" s="24" t="n">
+        <v/>
+      </c>
+      <c r="O18" s="24" t="str">
         <f aca="false">IF(N18="","",SIGN(H18)*MIN(ABS(H18),ABS(I18))-N18)</f>
-        <v>1.5446039038792</v>
+        <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
         <v>487</v>
       </c>
-      <c r="B19" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="C19" s="19" t="n">
-        <v>45</v>
-      </c>
-      <c r="D19" s="19" t="n">
-        <v>55.4</v>
-      </c>
-      <c r="E19" s="19" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="F19" s="19" t="n">
-        <v>36.3</v>
-      </c>
-      <c r="G19" s="19" t="n">
-        <v>35.6</v>
-      </c>
-      <c r="H19" s="24" t="n">
+      <c r="B19" s="14"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="24" t="str">
         <f aca="false">IF(COUNT(D19:E19)=0,"",AVERAGE(D19:E19))</f>
-        <v>55.05</v>
-      </c>
-      <c r="I19" s="24" t="n">
+        <v/>
+      </c>
+      <c r="I19" s="24" t="str">
         <f aca="false">IF(COUNT(F19:G19)=0,"",AVERAGE(F19:G19))</f>
-        <v>35.95</v>
-      </c>
-      <c r="J19" s="24" t="n">
+        <v/>
+      </c>
+      <c r="J19" s="24" t="str">
         <f aca="false">IF(OR(H19="",I19=""),"",IF(ABS(H19+I19)&lt;0.05,0,DEGREES(ATAN(2/(1/TAN(RADIANS(H19))+1/TAN(RADIANS(I19)))))))</f>
-        <v>43.9067346050426</v>
-      </c>
-      <c r="K19" s="24" t="n">
+        <v/>
+      </c>
+      <c r="K19" s="24" t="str">
         <f aca="false">IF(OR(J19="",C19=""),"",J19-C19)</f>
-        <v>-1.09326539495743</v>
-      </c>
-      <c r="L19" s="24" t="n">
+        <v/>
+      </c>
+      <c r="L19" s="24" t="str">
         <f aca="false">IF(COUNT(D19:E19)&lt;2,"",D19-E19)</f>
-        <v>0.699999999999996</v>
-      </c>
-      <c r="M19" s="24" t="n">
+        <v/>
+      </c>
+      <c r="M19" s="24" t="str">
         <f aca="false">IF(COUNT(F19:G19)&lt;2,"",F19-G19)</f>
-        <v>0.699999999999996</v>
-      </c>
-      <c r="N19" s="24" t="n">
+        <v/>
+      </c>
+      <c r="N19" s="24" t="str">
         <f aca="false">IF(OR(H19="",I19=""),"",IF(ABS(H19)&lt;0.05,0,SIGN(H19)*DEGREES(ATAN(1/(1/TAN(RADIANS(MAX(ABS(H19),ABS(I19))))+$B$6/$B$5)))))</f>
-        <v>37.9926450030618</v>
-      </c>
-      <c r="O19" s="24" t="n">
+        <v/>
+      </c>
+      <c r="O19" s="24" t="str">
         <f aca="false">IF(N19="","",SIGN(H19)*MIN(ABS(H19),ABS(I19))-N19)</f>
-        <v>-2.04264500306175</v>
+        <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16147,9 +16041,9 @@
       <c r="A22" s="18" t="s">
         <v>489</v>
       </c>
-      <c r="C22" s="30" t="n">
+      <c r="C22" s="30" t="str">
         <f aca="false">IF(COUNT(L11:M19)=0,"",MAX(MAX(L11:M19),-MIN(L11:M19)))</f>
-        <v>0.699999999999996</v>
+        <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16158,7 +16052,7 @@
       </c>
       <c r="C23" s="30" t="n">
         <f aca="false">IF(COUNT(K11:K19)=0,"",SUMPRODUCT(ABS(N(+K11:K19)))/COUNT(K11:K19))</f>
-        <v>1.91809409898476</v>
+        <v>4.295528035620938</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16167,7 +16061,7 @@
       </c>
       <c r="C24" s="30" t="n">
         <f aca="false">IF(COUNT(K11:K19)=0,"",MAX(MAX(K11:K19),-MIN(K11:K19)))</f>
-        <v>3.90702532245617</v>
+        <v>8.108425649729895</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add the measured grip and tipping limits (T08)
Lateral mu is 0.98 clean and after three runs, so dust costs no measurable
grip. The front wheels cannot be blocked, so the longitudinal test stands
front downhill on the blocked rear axle; with the load transfer this gives
mu 1.18 (less certain) and a traction limit of about 9 m/s^2, at least
6.7 m/s^2 with the lateral mu. The robot slides at 9.6 m/s^2 and would tip
at 12.5 m/s^2. The LEGO comparison was not measured and is removed.

Workbook: CoG from the sum of the axle loads with the effective wheel
radius, as in the journal, and the cached values refreshed. Validation
status: only the wheels, camera and holder were weighed singly.
</commit_message>
<xml_diff>
--- a/docs/data/manual/mobility_measurements.xlsx
+++ b/docs/data/manual/mobility_measurements.xlsx
@@ -162,7 +162,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="664">
   <si>
     <t xml:space="preserve">Test Plan &amp; Measurement Series, Chapter 2 – Napoleon (Chassis Vertikal v36/v38)</t>
   </si>
@@ -2000,16 +2000,16 @@
     <t xml:space="preserve">Condition</t>
   </si>
   <si>
-    <t xml:space="preserve">Sliding angle α [°] (5 measurements →)</t>
+    <t xml:space="preserve">Sliding angle α [°] (one column per run →)</t>
   </si>
   <si>
     <t xml:space="preserve">Mean α [°]</t>
   </si>
   <si>
-    <t xml:space="preserve">μ = tan α</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Longitudinal (wheels blocked)</t>
+    <t xml:space="preserve">μ (formula see note)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longitudinal (front downhill, rear wheels blocked)</t>
   </si>
   <si>
     <t xml:space="preserve">clean</t>
@@ -2142,6 +2142,18 @@
   </si>
   <si>
     <t xml:space="preserve">63.2 % crossing [s]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effective wheel radius r_eff [mm]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Encoder calibration T04 (30.0 mm effective diameter); used for z_CoG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not measured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measured 02.10.2026, 3 runs each; "clean" = tyres washed with water, "after 3 runs" = 3 runs on the mat without cleaning. Lateral: μ = tan α. Longitudinal: the front wheels roll freely, only the blocked rear axle holds the robot: μ = L·tan α / (l_f − h·tan α), l_f = L − x_CoG.</t>
   </si>
 </sst>
 </file>
@@ -13559,6 +13571,17 @@
         <v>361</v>
       </c>
     </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>660</v>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>661</v>
+      </c>
+    </row>
     <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
         <v>362</v>
@@ -15345,7 +15368,7 @@
       </c>
       <c r="B62" s="24" t="n">
         <f aca="false">IF(OR(B56="",B57="",B55=""),"",B56+B57-B55)</f>
-        <v>0.400000000000091</v>
+        <v>-7.0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15353,8 +15376,8 @@
         <v>431</v>
       </c>
       <c r="B63" s="24" t="n">
-        <f aca="false">IF(OR(B56="",B55=""),"",$B$8*B56/B55)</f>
-        <v>59.5192073700678</v>
+        <f aca="false">IF(OR(B56="",B57=""),"",$B$8*B56/(B56+B57))</f>
+        <v>56.72538860103627</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15363,7 +15386,7 @@
       </c>
       <c r="B64" s="24" t="n">
         <f aca="false">IF(OR(B58="",B59=""),"",$B$9*(B58/(B58+B59)-0.5))</f>
-        <v>2.71033043478261</v>
+        <v>-0.9138169257340238</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15372,7 +15395,7 @@
       </c>
       <c r="B65" s="30" t="n">
         <f aca="false">IF(B60="","",DEGREES(ASIN(B60/$B$8)))</f>
-        <v>14.187627613403</v>
+        <v>23.088772437010103</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15380,8 +15403,8 @@
         <v>433</v>
       </c>
       <c r="B66" s="24" t="n">
-        <f aca="false">IF(OR(B61="",B56="",B60="",B55=""),"",$B$10+$B$8*(B61-B56)/(B55*TAN(RADIANS(B65))))</f>
-        <v>31.2886629259024</v>
+        <f aca="false">IF(OR(B61="",B56="",B57="",B60=""),"",$B$11+$B$8*(B61-B56)/((B56+B57)*TAN(RADIANS(B65))))</f>
+        <v>37.728162360345706</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15413,11 +15436,11 @@
       </c>
       <c r="C70" s="24" t="n">
         <f aca="false">B55</f>
-        <v>575.3</v>
+        <v>586.0</v>
       </c>
       <c r="D70" s="24" t="n">
         <f aca="false">IF(OR(B70="",C70="",B70=0),"",C70-B70)</f>
-        <v>2.29999999999995</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15430,11 +15453,11 @@
       </c>
       <c r="C71" s="24" t="n">
         <f aca="false">B63</f>
-        <v>59.5192073700678</v>
+        <v>56.72538860103627</v>
       </c>
       <c r="D71" s="24" t="n">
         <f aca="false">IF(OR(B71="",C71="",B71=0),"",C71-B71)</f>
-        <v>-1.40527605052556</v>
+        <v>-4.199094819557125</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15447,11 +15470,11 @@
       </c>
       <c r="C72" s="24" t="n">
         <f aca="false">B64</f>
-        <v>2.71033043478261</v>
+        <v>-0.9138169257340238</v>
       </c>
       <c r="D72" s="24" t="n">
         <f aca="false">IF(OR(B72="",C72="",B72=0),"",C72-B72)</f>
-        <v>-0.565500280749676</v>
+        <v>-4.189647641266314</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15464,11 +15487,11 @@
       </c>
       <c r="C73" s="24" t="n">
         <f aca="false">B66</f>
-        <v>31.2886629259024</v>
+        <v>37.728162360345706</v>
       </c>
       <c r="D73" s="24" t="n">
         <f aca="false">IF(OR(B73="",C73="",B73=0),"",C73-B73)</f>
-        <v>1.08870830112057</v>
+        <v>7.528207735563807</v>
       </c>
     </row>
   </sheetData>
@@ -19164,7 +19187,7 @@
       </c>
       <c r="B11" s="30" t="n">
         <f aca="false">IF(Mass_CoG!B55&lt;&gt;"",Mass_CoG!B55,Mass_CoG!C47)</f>
-        <v>575.3</v>
+        <v>586.0</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>559</v>
@@ -19176,7 +19199,7 @@
       </c>
       <c r="B12" s="30" t="n">
         <f aca="false">IF(Mass_CoG!B63&lt;&gt;"",Mass_CoG!B63,Mass_CoG!C48)</f>
-        <v>59.5192073700678</v>
+        <v>56.72538860103627</v>
       </c>
       <c r="C12" s="20" t="s">
         <v>560</v>
@@ -19188,7 +19211,7 @@
       </c>
       <c r="B13" s="30" t="n">
         <f aca="false">IF(Mass_CoG!B66&lt;&gt;"",Mass_CoG!B66,Mass_CoG!C50)</f>
-        <v>31.2886629259024</v>
+        <v>37.728162360345706</v>
       </c>
       <c r="C13" s="20" t="s">
         <v>560</v>
@@ -19210,7 +19233,7 @@
       </c>
       <c r="B15" s="30" t="n">
         <f aca="false">Grip_Tipping!C12</f>
-        <v>0.8779031807736</v>
+        <v>1.1769754505259147</v>
       </c>
       <c r="C15" s="20" t="s">
         <v>562</v>
@@ -19307,7 +19330,7 @@
       </c>
       <c r="B27" s="28" t="n">
         <f aca="false">IF(OR(B12="",B14=""),"",1-B12/B14)</f>
-        <v>0.416478359116982</v>
+        <v>0.4438687392055267</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19316,7 +19339,7 @@
       </c>
       <c r="B28" s="30" t="n">
         <f aca="false">IF(OR(B15="",B12="",B13=""),"",B15*9.81*(1-B12/B14)/(1-B15*B13/B14))</f>
-        <v>4.9087158648216</v>
+        <v>9.076267185742973</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19713,27 +19736,23 @@
         <v>616</v>
       </c>
       <c r="C5" s="19" t="n">
-        <v>40.9</v>
+        <v>21</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>41.2</v>
+        <v>20</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="G5" s="19" t="n">
-        <v>41.4</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
       <c r="H5" s="24" t="n">
         <f aca="false">IF(COUNT(C5:G5)=0,"",AVERAGE(C5:G5))</f>
-        <v>41.28</v>
+        <v>20.0</v>
       </c>
       <c r="I5" s="30" t="n">
-        <f aca="false">IF(H5="","",TAN(RADIANS(H5)))</f>
-        <v>0.8779031807736</v>
+        <f aca="false">IF(H5="","",Drivetrain!$B$14*TAN(RADIANS(H5))/(Drivetrain!$B$14-Drivetrain!$B$12-Drivetrain!$B$13*TAN(RADIANS(H5))))</f>
+        <v>1.1769754505259147</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19744,27 +19763,23 @@
         <v>617</v>
       </c>
       <c r="C6" s="19" t="n">
-        <v>34.1</v>
+        <v>21</v>
       </c>
       <c r="D6" s="19" t="n">
-        <v>35.2</v>
+        <v>22</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>35</v>
-      </c>
-      <c r="F6" s="19" t="n">
-        <v>35.1</v>
-      </c>
-      <c r="G6" s="19" t="n">
-        <v>33.3</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
       <c r="H6" s="24" t="n">
         <f aca="false">IF(COUNT(C6:G6)=0,"",AVERAGE(C6:G6))</f>
-        <v>34.54</v>
+        <v>21.333333333333332</v>
       </c>
       <c r="I6" s="30" t="n">
-        <f aca="false">IF(H6="","",TAN(RADIANS(H6)))</f>
-        <v>0.688309349985208</v>
+        <f aca="false">IF(H6="","",Drivetrain!$B$14*TAN(RADIANS(H6))/(Drivetrain!$B$14-Drivetrain!$B$12-Drivetrain!$B$13*TAN(RADIANS(H6))))</f>
+        <v>1.3044163524448116</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19775,27 +19790,23 @@
         <v>616</v>
       </c>
       <c r="C7" s="19" t="n">
-        <v>44.3</v>
+        <v>43</v>
       </c>
       <c r="D7" s="19" t="n">
-        <v>44.2</v>
+        <v>45</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>45.3</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <v>43.8</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
       <c r="H7" s="24" t="n">
         <f aca="false">IF(COUNT(C7:G7)=0,"",AVERAGE(C7:G7))</f>
-        <v>44.6</v>
+        <v>44.333333333333336</v>
       </c>
       <c r="I7" s="30" t="n">
         <f aca="false">IF(H7="","",TAN(RADIANS(H7)))</f>
-        <v>0.986133944044009</v>
+        <v>0.9769955737951757</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19806,27 +19817,23 @@
         <v>617</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>35.6</v>
+        <v>47</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>35.7</v>
+        <v>43</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="F8" s="19" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="G8" s="19" t="n">
-        <v>36.7</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
       <c r="H8" s="24" t="n">
         <f aca="false">IF(COUNT(C8:G8)=0,"",AVERAGE(C8:G8))</f>
-        <v>36.06</v>
+        <v>44.333333333333336</v>
       </c>
       <c r="I8" s="30" t="n">
         <f aca="false">IF(H8="","",TAN(RADIANS(H8)))</f>
-        <v>0.728143722319513</v>
+        <v>0.9769955737951757</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19836,28 +19843,25 @@
       <c r="B9" s="18" t="s">
         <v>616</v>
       </c>
-      <c r="C9" s="19" t="n">
-        <v>30.4</v>
-      </c>
-      <c r="D9" s="19" t="n">
-        <v>29.8</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>30.7</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="H9" s="24" t="n">
+      <c r="C9" s="19" t="s">
+        <v>662</v>
+      </c>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="24" t="str">
         <f aca="false">IF(COUNT(C9:G9)=0,"",AVERAGE(C9:G9))</f>
-        <v>30.58</v>
-      </c>
-      <c r="I9" s="30" t="n">
+        <v/>
+      </c>
+      <c r="I9" s="30" t="str">
         <f aca="false">IF(H9="","",TAN(RADIANS(H9)))</f>
-        <v>0.590927296290316</v>
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19871,7 +19875,7 @@
       </c>
       <c r="C12" s="30" t="n">
         <f aca="false">I5</f>
-        <v>0.8779031807736</v>
+        <v>1.1769754505259147</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19880,7 +19884,7 @@
       </c>
       <c r="C13" s="30" t="n">
         <f aca="false">I7</f>
-        <v>0.986133944044009</v>
+        <v>0.9769955737951757</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19889,7 +19893,7 @@
       </c>
       <c r="C14" s="24" t="n">
         <f aca="false">Drivetrain!B13</f>
-        <v>31.2886629259024</v>
+        <v>37.728162360345706</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19907,7 +19911,7 @@
       </c>
       <c r="C17" s="24" t="n">
         <f aca="false">IF(OR(C14="",C14=0),"",9.81*C15/2/C14)</f>
-        <v>15.0808937127629</v>
+        <v>12.506864116338486</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19916,7 +19920,7 @@
       </c>
       <c r="C18" s="24" t="n">
         <f aca="false">IF(C13="","",C13*9.81)</f>
-        <v>9.67397399107173</v>
+        <v>9.584326578930673</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19934,7 +19938,7 @@
       </c>
       <c r="C20" s="24" t="n">
         <f aca="false">IF(OR(C17="",C18="",C18=0),"",C17/C18)</f>
-        <v>1.5589140229942</v>
+        <v>1.304928834941044</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -19958,7 +19962,7 @@
       </c>
       <c r="C23" s="30" t="n">
         <f aca="false">IF(C13="","",SQRT(C13*9.81*A23/1000))</f>
-        <v>0.983563622297599</v>
+        <v>0.9789957394662488</v>
       </c>
       <c r="D23" s="28" t="n">
         <f aca="false">$C$15/(2*A23)</f>
@@ -19975,7 +19979,7 @@
       </c>
       <c r="C24" s="30" t="n">
         <f aca="false">IF(C13="","",SQRT(C13*9.81*A24/1000))</f>
-        <v>1.20461450209632</v>
+        <v>1.1990200110255045</v>
       </c>
       <c r="D24" s="28" t="n">
         <f aca="false">$C$15/(2*A24)</f>
@@ -19992,7 +19996,7 @@
       </c>
       <c r="C25" s="30" t="n">
         <f aca="false">IF(C13="","",SQRT(C13*9.81*A25/1000))</f>
-        <v>1.39096901411007</v>
+        <v>1.384509052258646</v>
       </c>
       <c r="D25" s="28" t="n">
         <f aca="false">$C$15/(2*A25)</f>
@@ -20009,7 +20013,7 @@
       </c>
       <c r="C26" s="30" t="n">
         <f aca="false">IF(C13="","",SQRT(C13*9.81*A26/1000))</f>
-        <v>1.70358216629593</v>
+        <v>1.6956703611490065</v>
       </c>
       <c r="D26" s="28" t="n">
         <f aca="false">$C$15/(2*A26)</f>
@@ -20026,7 +20030,7 @@
       </c>
       <c r="C27" s="30" t="n">
         <f aca="false">IF(C13="","",SQRT(C13*9.81*A27/1000))</f>
-        <v>2.19931511965336</v>
+        <v>2.189101023129206</v>
       </c>
       <c r="D27" s="28" t="n">
         <f aca="false">$C$15/(2*A27)</f>
@@ -20043,7 +20047,7 @@
       </c>
       <c r="C28" s="30" t="n">
         <f aca="false">IF(C13="","",SQRT(C13*9.81*A28/1000))</f>
-        <v>2.69359991336943</v>
+        <v>2.681090251035575</v>
       </c>
       <c r="D28" s="28" t="n">
         <f aca="false">$C$15/(2*A28)</f>
@@ -20060,7 +20064,7 @@
       </c>
       <c r="C29" s="30" t="n">
         <f aca="false">IF(C13="","",SQRT(C13*9.81*A29/1000))</f>
-        <v>3.11030127014599</v>
+        <v>3.0958563563141417</v>
       </c>
       <c r="D29" s="28" t="n">
         <f aca="false">$C$15/(2*A29)</f>

</xml_diff>